<commit_message>
Update tracker spreadsheet with Vercel links for gluten-free guide and completed blog articles
</commit_message>
<xml_diff>
--- a/Pragmatic Nutrition - Page Tracker.xlsx
+++ b/Pragmatic Nutrition - Page Tracker.xlsx
@@ -1092,7 +1092,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:5176/gluten-free-diet</t>
+          <t>https://pragmatic-nutritionist.vercel.app/gluten-free-diet</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
@@ -1159,7 +1159,11 @@
       <c r="C43" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="D43" s="7" t="n"/>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/best-sports-nutritionist-in-chennai</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1178,7 +1182,11 @@
       <c r="C44" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="D44" s="7" t="n"/>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/genetic-methylation-test</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1197,7 +1205,11 @@
       <c r="C45" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="D45" s="7" t="n"/>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/glp-1-side-effects</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1216,7 +1228,11 @@
       <c r="C46" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="D46" s="7" t="n"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/l-theanine-supplement</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1235,7 +1251,11 @@
       <c r="C47" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/low-stomach-acid-symptoms</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1254,7 +1274,11 @@
       <c r="C48" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="D48" s="7" t="n"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/mcas</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1273,7 +1297,11 @@
       <c r="C49" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="D49" s="7" t="n"/>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/psyllium-husk-benefits-side-effects</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1292,7 +1320,11 @@
       <c r="C50" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="D50" s="7" t="n"/>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/runners-stomach</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1311,7 +1343,11 @@
       <c r="C51" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="D51" s="7" t="n"/>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/saffron-for-adhd</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1330,7 +1366,11 @@
       <c r="C52" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="D52" s="7" t="n"/>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/vagus-nerve</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -1349,7 +1389,11 @@
       <c r="C53" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="D53" s="7" t="n"/>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>https://pragmatic-nutritionist.vercel.app/blog/what-is-ibd-ibd-vs-ibs</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>Oct 29</t>
@@ -6977,6 +7021,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId249"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId250"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId263"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>